<commit_message>
document which details all the solvent/electrolyte properties
</commit_message>
<xml_diff>
--- a/all_props.xlsx
+++ b/all_props.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/vm5_ornl_gov/Documents/Projects/MixedSolvents/InputData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{F4EA342B-8340-4219-8C67-3E8FFC6A3338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA4F77E9-929C-47C1-BC73-515F30126DB4}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{F4EA342B-8340-4219-8C67-3E8FFC6A3338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C89A2E0-E712-4B1F-8869-AE644680B3B6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DC0318B6-9308-42E5-B13E-10902EEE5460}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DC0318B6-9308-42E5-B13E-10902EEE5460}"/>
   </bookViews>
   <sheets>
     <sheet name="PropertyData" sheetId="1" r:id="rId1"/>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
-  <si>
-    <t>Molecular details</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
   <si>
     <t>Abbreviation</t>
   </si>
@@ -135,7 +132,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -143,25 +140,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -176,12 +161,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,83 +497,94 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CDF8C01-F29C-477B-9213-4C066B6F0425}">
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>18.015000000000001</v>
+      </c>
+      <c r="E2">
+        <v>0.997</v>
+      </c>
+      <c r="F2">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>28</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>23</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D3">
-        <v>18.015000000000001</v>
+        <v>62.07</v>
       </c>
       <c r="E3">
-        <v>0.997</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="F3">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C4">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>62.07</v>
+        <v>32.04</v>
       </c>
       <c r="E4">
-        <v>1.1100000000000001</v>
+        <v>0.79100000000000004</v>
       </c>
       <c r="F4">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -600,39 +592,39 @@
         <v>17</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="D5">
-        <v>32.04</v>
+        <v>222.28</v>
       </c>
       <c r="E5">
-        <v>0.79100000000000004</v>
+        <v>1.0089999999999999</v>
       </c>
       <c r="F5">
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C6">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>222.28</v>
+        <v>72.11</v>
       </c>
       <c r="E6">
-        <v>1.0089999999999999</v>
+        <v>0.88800000000000001</v>
       </c>
       <c r="F6">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -640,19 +632,19 @@
         <v>9</v>
       </c>
       <c r="C7">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7">
-        <v>72.11</v>
+        <v>73.09</v>
       </c>
       <c r="E7">
-        <v>0.88800000000000001</v>
+        <v>0.94399999999999995</v>
       </c>
       <c r="F7">
         <v>2250</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -660,39 +652,39 @@
         <v>10</v>
       </c>
       <c r="C8">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D8">
-        <v>73.09</v>
+        <v>41.052999999999997</v>
       </c>
       <c r="E8">
-        <v>0.94399999999999995</v>
+        <v>0.78600000000000003</v>
       </c>
       <c r="F8">
-        <v>2250</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>6</v>
       </c>
-      <c r="D9">
-        <v>41.052999999999997</v>
-      </c>
-      <c r="E9">
-        <v>0.78600000000000003</v>
-      </c>
-      <c r="F9">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D10">
+        <v>151.91</v>
+      </c>
+      <c r="E10">
+        <v>3.65</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -700,19 +692,19 @@
         <v>12</v>
       </c>
       <c r="C11">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D11">
-        <v>151.91</v>
+        <v>126.75</v>
       </c>
       <c r="E11">
-        <v>3.65</v>
+        <v>3.16</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -720,19 +712,19 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D12">
-        <v>126.75</v>
+        <v>142.04</v>
       </c>
       <c r="E12">
-        <v>3.16</v>
+        <v>2.6640000000000001</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -740,19 +732,19 @@
         <v>14</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <v>142.04</v>
+        <v>58.44</v>
       </c>
       <c r="E13">
-        <v>2.6640000000000001</v>
+        <v>2.165</v>
       </c>
       <c r="F13">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -760,79 +752,79 @@
         <v>15</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D14">
-        <v>58.44</v>
+        <v>98.08</v>
       </c>
       <c r="E14">
-        <v>2.165</v>
+        <v>1.83</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15">
-        <v>7</v>
-      </c>
-      <c r="D15">
-        <v>98.08</v>
-      </c>
-      <c r="E15">
-        <v>1.83</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>55.844999999999999</v>
+      </c>
+      <c r="E16">
+        <v>7.7839999999999998</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D17">
-        <v>55.844999999999999</v>
+        <v>96.064999999999998</v>
       </c>
       <c r="E17">
-        <v>7.7839999999999998</v>
+        <v>2.67</v>
       </c>
       <c r="F17">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C18">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D18">
-        <v>96.064999999999998</v>
+        <v>22.99</v>
       </c>
       <c r="E18">
-        <v>2.67</v>
+        <v>0.96799999999999997</v>
       </c>
       <c r="F18">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -843,39 +835,16 @@
         <v>1</v>
       </c>
       <c r="D19">
-        <v>22.99</v>
+        <v>35.450000000000003</v>
       </c>
       <c r="E19">
-        <v>0.96799999999999997</v>
+        <v>1.56</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20">
-        <v>35.450000000000003</v>
-      </c>
-      <c r="E20">
-        <v>1.56</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>